<commit_message>
Switch chunking to whole articles and clean the Qistas watermark
Phase 12a: production chunking moves from 531 clause-level fragments to
whole articles. Clause chunks were semantically incomplete on their own
("Pension stipulated in Paragraph (a) ... shall be increased by 0.5%"
never names the pension), and six near-identical fragments of SSL 71
crowded out the correct article entirely on q22. Whole articles won every
retrieval metric: same-language recall@10 0.969 -> 1.000.

Also removes a PDF watermark ("حقوق قسطاس للتقنيات القانونية") that
extraction had read as body text. In Article 65 it was spliced
mid-sentence, so it damaged the embedding, the BM25 term statistics, and
the context handed to the generator all at once.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/0. cleaned_data/Knowledgebase/worklaw_ar_articles.xlsx
+++ b/0. cleaned_data/Knowledgebase/worklaw_ar_articles.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,8 +444,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -461,8 +463,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>2</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,8 +517,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>3</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -537,8 +543,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>4</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -561,8 +569,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -582,8 +592,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>6</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -604,8 +616,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>7</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -626,8 +640,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>8</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -650,8 +666,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>9</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -676,8 +694,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>10</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -700,8 +720,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>11</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -718,8 +740,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>12</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -764,8 +788,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>13</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -790,8 +816,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>14</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -815,8 +843,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>15</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -851,8 +881,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>16</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -874,8 +906,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>17</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -897,8 +931,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>18</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,8 +955,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>19</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -947,8 +985,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>20</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -967,8 +1007,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>21</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -988,8 +1030,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>22</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1009,8 +1053,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>23</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1036,8 +1082,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>24</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1058,8 +1106,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>25</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1082,8 +1132,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>26</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1108,8 +1160,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>27</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1136,8 +1190,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>28</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1168,8 +1224,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B30" t="n">
-        <v>29</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1204,8 +1262,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>30</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1227,8 +1287,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>31</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1260,8 +1322,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>32</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1285,13 +1349,14 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>33</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>المادة (33): أنظمة صناديق الادخار أو التوفير أو التقاعد
-٣٩ / ١١
 أ - بالإضافة لمكافأة نهاية الخدمة يحق للعامل الجامع أنظمة خاصة للمؤسسة التي يعمل فيها تتعلق بصناديق الإدخار أو التوفير أو
 التقاعد أو أي صندوق آخر مماثل الحصول على جميع الاستحقاقات الممنوحة له بموجب هذه الأنظمة في حالة انتهاء الخدمة .
 ب - تعتمد الأنظمة الخاصة بالصناديق المنصوص عليها في الفقرة (أ) من هذه المادة من قبل الوزير .
@@ -1312,8 +1377,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B35" t="n">
-        <v>34</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1334,8 +1401,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>35</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1359,8 +1428,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>36</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1384,14 +1455,14 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>37</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
           <t>المادة (37): مدة عقد التدريب
-قسطاس للتقنيات القانونية
-٣٩ / ١٢
 تحدد في عقد التدريب مدته ومراحله المتعاقبة والأجور المستحقة للمتدرب في كل مرحلة ويجب أن لا يقل الأجر في المرحلة الأخيرة عن
 الحد الأدنى للأجر المعطى لعمل مماثل وأن يكون تحديده بحال من الأحوال على أساس القطعة أو الإنتاج وينظم التدريب وفق البرامج
 التي تحددها مؤسسة التدريب المهني بتعليمات تصدرها لهذا الغرض وتنشر في الجريدة الرسمية.</t>
@@ -1409,8 +1480,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>38</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1437,8 +1510,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>39</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1462,8 +1537,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B41" t="n">
-        <v>40</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1487,8 +1564,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B42" t="n">
-        <v>41</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1512,8 +1591,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B43" t="n">
-        <v>42</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1548,8 +1629,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>43</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1577,8 +1660,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>44</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1603,8 +1688,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B46" t="n">
-        <v>45</v>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1625,8 +1712,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B47" t="n">
-        <v>46</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1649,8 +1738,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>47</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1679,8 +1770,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B49" t="n">
-        <v>48</v>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1709,8 +1802,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B50" t="n">
-        <v>49</v>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1733,8 +1828,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>50</v>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1756,8 +1853,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B52" t="n">
-        <v>51</v>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1783,8 +1882,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B53" t="n">
-        <v>52</v>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1809,8 +1910,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B54" t="n">
-        <v>53</v>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1832,8 +1935,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B55" t="n">
-        <v>54</v>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1897,8 +2002,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B56" t="n">
-        <v>55</v>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1918,8 +2025,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B57" t="n">
-        <v>56</v>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1940,8 +2049,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B58" t="n">
-        <v>57</v>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1963,8 +2074,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B59" t="n">
-        <v>58</v>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1984,8 +2097,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B60" t="n">
-        <v>59</v>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -2006,8 +2121,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B61" t="n">
-        <v>60</v>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -2028,8 +2145,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B62" t="n">
-        <v>61</v>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -2054,8 +2173,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B63" t="n">
-        <v>62</v>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2071,8 +2192,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B64" t="n">
-        <v>63</v>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2089,8 +2212,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B65" t="n">
-        <v>64</v>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -2106,15 +2231,16 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B66" t="n">
-        <v>65</v>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
           <t>المادة (65): الإجازات المرضية تاريخ السريان ١٦-٠٥-٢٠١٩
 لكل عامل الحق في إجازة مرضية مدتها أربعة عشر يوماً خلال السنة الواحدة بأجر كامل بناء على تقرير من الطبيب المعتمد من قبل
 المؤسسة ، ويجوز تمديدها لمدة أربعة عشر يوماً أخرى بأجر كامل إذا كان نزيل أحد المستشفيات بناء على تقرير من الطبيب المعتمد
-حقوق قسطاس للتقنيات القانونية
 من قبل المؤسسات التي يقل عدد عمالها عن عشرين عاملاً، أما المؤسسات التي يزيد عدد عمالها على عشرين عاملاً فيتم اعتماد لجنة
 طبية خاصة لغايات اعتماد التقارير الطبية.</t>
         </is>
@@ -2127,8 +2253,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B67" t="n">
-        <v>66</v>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -2154,8 +2282,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B68" t="n">
-        <v>67</v>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -2177,8 +2307,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B69" t="n">
-        <v>68</v>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2199,8 +2331,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B70" t="n">
-        <v>69</v>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2221,8 +2355,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B71" t="n">
-        <v>70</v>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2243,8 +2379,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B72" t="n">
-        <v>71</v>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2265,8 +2403,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B73" t="n">
-        <v>72</v>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2290,8 +2430,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B74" t="n">
-        <v>73</v>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2312,8 +2454,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B75" t="n">
-        <v>74</v>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2334,8 +2478,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B76" t="n">
-        <v>75</v>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2358,8 +2504,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B77" t="n">
-        <v>76</v>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2383,8 +2531,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B78" t="n">
-        <v>77</v>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2410,8 +2560,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B79" t="n">
-        <v>78</v>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2439,8 +2591,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B80" t="n">
-        <v>79</v>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2462,8 +2616,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B81" t="n">
-        <v>80</v>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2484,8 +2640,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B82" t="n">
-        <v>81</v>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2507,8 +2665,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B83" t="n">
-        <v>82</v>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2531,8 +2691,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B84" t="n">
-        <v>83</v>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2554,8 +2716,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B85" t="n">
-        <v>84</v>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2580,8 +2744,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B86" t="n">
-        <v>85</v>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2604,8 +2770,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B87" t="n">
-        <v>86</v>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2625,8 +2793,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B88" t="n">
-        <v>87</v>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2647,8 +2817,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B89" t="n">
-        <v>88</v>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2668,8 +2840,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B90" t="n">
-        <v>89</v>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2690,8 +2864,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B91" t="n">
-        <v>90</v>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2720,8 +2896,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B92" t="n">
-        <v>91</v>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2742,8 +2920,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B93" t="n">
-        <v>92</v>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2770,8 +2950,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B94" t="n">
-        <v>93</v>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2797,8 +2979,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B95" t="n">
-        <v>94</v>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2827,8 +3011,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B96" t="n">
-        <v>95</v>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2850,8 +3036,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B97" t="n">
-        <v>96</v>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2872,8 +3060,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B98" t="n">
-        <v>97</v>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -2899,8 +3089,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B99" t="n">
-        <v>98</v>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -2935,8 +3127,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B100" t="n">
-        <v>99</v>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -2963,8 +3157,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B101" t="n">
-        <v>100</v>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -2995,8 +3191,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B102" t="n">
-        <v>101</v>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -3020,8 +3218,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B103" t="n">
-        <v>102</v>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -3049,8 +3249,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B104" t="n">
-        <v>103</v>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -3077,8 +3279,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B105" t="n">
-        <v>104</v>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -3099,8 +3303,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B106" t="n">
-        <v>105</v>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -3121,8 +3327,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B107" t="n">
-        <v>106</v>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -3144,8 +3352,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B108" t="n">
-        <v>107</v>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -3166,8 +3376,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B109" t="n">
-        <v>108</v>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -3194,8 +3406,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B110" t="n">
-        <v>109</v>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -3219,8 +3433,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B111" t="n">
-        <v>110</v>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -3243,8 +3459,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B112" t="n">
-        <v>111</v>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -3265,8 +3483,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B113" t="n">
-        <v>112</v>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -3286,8 +3506,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B114" t="n">
-        <v>113</v>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -3308,8 +3530,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B115" t="n">
-        <v>114</v>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -3331,8 +3555,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B116" t="n">
-        <v>115</v>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -3353,8 +3579,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B117" t="n">
-        <v>116</v>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -3380,8 +3608,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B118" t="n">
-        <v>117</v>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -3403,8 +3633,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B119" t="n">
-        <v>118</v>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -3429,8 +3661,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B120" t="n">
-        <v>119</v>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
@@ -3454,8 +3688,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B121" t="n">
-        <v>120</v>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -3476,8 +3712,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B122" t="n">
-        <v>121</v>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -3504,8 +3742,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B123" t="n">
-        <v>122</v>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -3530,8 +3770,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B124" t="n">
-        <v>123</v>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -3551,8 +3793,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B125" t="n">
-        <v>124</v>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
@@ -3580,8 +3824,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B126" t="n">
-        <v>125</v>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
@@ -3603,8 +3849,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B127" t="n">
-        <v>126</v>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -3626,8 +3874,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B128" t="n">
-        <v>127</v>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>127</t>
+        </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
@@ -3648,8 +3898,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B129" t="n">
-        <v>128</v>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -3672,8 +3924,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B130" t="n">
-        <v>129</v>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -3694,8 +3948,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B131" t="n">
-        <v>130</v>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
@@ -3715,8 +3971,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B132" t="n">
-        <v>131</v>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
@@ -3738,8 +3996,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B133" t="n">
-        <v>132</v>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
@@ -3762,8 +4022,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B134" t="n">
-        <v>133</v>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
@@ -3788,8 +4050,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B135" t="n">
-        <v>134</v>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>134</t>
+        </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
@@ -3808,8 +4072,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B136" t="n">
-        <v>135</v>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>135</t>
+        </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -3829,8 +4095,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B137" t="n">
-        <v>136</v>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -3849,8 +4117,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B138" t="n">
-        <v>137</v>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -3888,8 +4158,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B139" t="n">
-        <v>138</v>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -3912,8 +4184,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B140" t="n">
-        <v>139</v>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -3935,8 +4209,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B141" t="n">
-        <v>140</v>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -3956,8 +4232,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B142" t="n">
-        <v>141</v>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -3979,8 +4257,10 @@
           <t>Worklaw_Arabic_1996</t>
         </is>
       </c>
-      <c r="B143" t="n">
-        <v>142</v>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>

</xml_diff>